<commit_message>
Cover first-launch T&C and Privacy links, then hand run_all an offline relaunch.
The suite now walks both policy pages when the one-time card is up, dismisses cookies before capturing them, and force-relaunches after Airplane Mode so later tests start genuinely offline.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/testrail/spider_unity_cases.xlsx
+++ b/docs/testrail/spider_unity_cases.xlsx
@@ -190,6 +190,100 @@
     <row>
       <c t="inlineStr">
         <is>
+          <t xml:space="preserve">FL-04</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Launch - Terms &amp; Conditions link opens the terms page</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spider Solitaire Unity &gt; Launch</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Functional</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">High</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. Delete Spider and reinstall it, or otherwise reset it so the Terms &amp; Conditions card is on screen. Do not tap Continue yet.
+2. Tap the Terms &amp; Conditions link.
+3. If Accept All Cookies appears, tap it and wait for the cookie banner to disappear.
+4. Close the page or tap Back.</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. The card shows links for Terms &amp; Conditions and Privacy Policy.
+2. A terms web page opens, not the Privacy Policy page.
+3. The banner is gone and the Terms of Service heading is fully visible.
+4. The Terms &amp; Conditions card is still there. Do not tap Continue yet.</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Manual</t>
+        </is>
+      </c>
+    </row>
+    <row>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">FL-05</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Launch - Privacy Policy link opens the privacy page</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spider Solitaire Unity &gt; Launch</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Functional</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">High</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. On the same Terms &amp; Conditions card, tap Privacy Policy.
+2. If Accept All Cookies appears, tap it and wait for the cookie banner to disappear.
+3. Close the page or tap Back.</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. A privacy web page opens, not the Terms &amp; Conditions page.
+2. The banner is gone and the Privacy Notice heading is fully visible.
+3. The Terms &amp; Conditions card is still there. Continue is checked separately in FL-02.</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Manual</t>
+        </is>
+      </c>
+    </row>
+    <row>
+      <c t="inlineStr">
+        <is>
           <t xml:space="preserve">MM-01</t>
         </is>
       </c>
@@ -221,6 +315,48 @@
       <c t="inlineStr">
         <is>
           <t xml:space="preserve">1. Play, Stats, Options, Help, About, More Games, Choose Look, and the Spider logo are all on screen.</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Manual</t>
+        </is>
+      </c>
+    </row>
+    <row>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">ST-01</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Statistics - Opens from the main menu</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spider Solitaire Unity &gt; Statistics</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Functional</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Medium</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. From the main menu, tap Stats.</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. The Statistics screen opens. The header reads Statistics. The main menu is gone.</t>
         </is>
       </c>
       <c t="inlineStr">
@@ -276,6 +412,90 @@
     <row>
       <c t="inlineStr">
         <is>
+          <t xml:space="preserve">ST-04</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Statistics - Back returns to the main menu</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spider Solitaire Unity &gt; Statistics</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Functional</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Medium</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. From Statistics, tap Back.</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. The main menu is showing.</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Manual</t>
+        </is>
+      </c>
+    </row>
+    <row>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">OP-01</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Options - Opens from the main menu</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spider Solitaire Unity &gt; Options</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Functional</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Medium</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. From the main menu, tap Options.</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. The Options screen opens. The main menu is gone.</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Manual</t>
+        </is>
+      </c>
+    </row>
+    <row>
+      <c t="inlineStr">
+        <is>
           <t xml:space="preserve">OP-03</t>
         </is>
       </c>
@@ -492,6 +712,48 @@
     <row>
       <c t="inlineStr">
         <is>
+          <t xml:space="preserve">HP-01</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Help - Opens on Introduction</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spider Solitaire Unity &gt; Help</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Functional</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Medium</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. From the main menu, tap Help.</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. Help opens with the Introduction heading. The main menu is gone.</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Manual</t>
+        </is>
+      </c>
+    </row>
+    <row>
+      <c t="inlineStr">
+        <is>
           <t xml:space="preserve">HP-02</t>
         </is>
       </c>
@@ -536,6 +798,90 @@
     <row>
       <c t="inlineStr">
         <is>
+          <t xml:space="preserve">HP-03</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Help - Back returns to the main menu</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spider Solitaire Unity &gt; Help</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Functional</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Medium</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. From Help, tap Back.</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. The main menu is showing.</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Manual</t>
+        </is>
+      </c>
+    </row>
+    <row>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">AB-01</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">About - Opens from the About menu item</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spider Solitaire Unity &gt; About</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Functional</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Medium</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. From the main menu, tap About.</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. The About screen opens. You can see the copyright line.</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Manual</t>
+        </is>
+      </c>
+    </row>
+    <row>
+      <c t="inlineStr">
+        <is>
           <t xml:space="preserve">AB-03</t>
         </is>
       </c>
@@ -777,6 +1123,48 @@
       <c t="inlineStr">
         <is>
           <t xml:space="preserve">1. FreeCell and Spiderette come into view. The back button and instruction line at the top stay put.</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Manual</t>
+        </is>
+      </c>
+    </row>
+    <row>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">MG-03</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">More Games - Back returns to the main menu</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spider Solitaire Unity &gt; More Games</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Functional</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Medium</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. From the More Games page, tap Back.</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. The main menu is showing.</t>
         </is>
       </c>
       <c t="inlineStr">
@@ -1667,6 +2055,48 @@
       <c t="inlineStr">
         <is>
           <t xml:space="preserve">1. It says Easy level, matching the game you started, not some other level.</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Manual</t>
+        </is>
+      </c>
+    </row>
+    <row>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">VI-04</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Victory - Back returns to the main menu</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spider Solitaire Unity &gt; Victory</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Functional</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Medium</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. On Victory, tap the screen's own Back control — not New.</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. The main menu is showing. Leaving by Back leaves no game in progress.</t>
         </is>
       </c>
       <c t="inlineStr">
@@ -3209,6 +3639,48 @@
         <is>
           <t xml:space="preserve">1. Game Center opens, headed Achievements.
 2. Last Score is showing again.</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Manual</t>
+        </is>
+      </c>
+    </row>
+    <row>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">LS-05</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Last Score - Back returns to the main menu</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spider Solitaire Unity &gt; Last Score</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Functional</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Medium</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. From Last Score, tap Back until you reach the menu.</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. The main menu is showing.</t>
         </is>
       </c>
       <c t="inlineStr">
@@ -4029,6 +4501,300 @@
     <row>
       <c t="inlineStr">
         <is>
+          <t xml:space="preserve">FL-04</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Launch - Terms &amp; Conditions link opens the terms page</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spider Solitaire Unity &gt; Launch</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Functional</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">High</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Delete Spider and reinstall it, or otherwise reset it so the Terms &amp; Conditions card is on screen. Do not tap Continue yet.</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">The card shows links for Terms &amp; Conditions and Privacy Policy.</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Manual</t>
+        </is>
+      </c>
+    </row>
+    <row>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">FL-04</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Launch - Terms &amp; Conditions link opens the terms page</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spider Solitaire Unity &gt; Launch</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Functional</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">High</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tap the Terms &amp; Conditions link.</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">A terms web page opens, not the Privacy Policy page.</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Manual</t>
+        </is>
+      </c>
+    </row>
+    <row>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">FL-04</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Launch - Terms &amp; Conditions link opens the terms page</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spider Solitaire Unity &gt; Launch</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Functional</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">High</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">If Accept All Cookies appears, tap it and wait for the cookie banner to disappear.</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">The banner is gone and the Terms of Service heading is fully visible.</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Manual</t>
+        </is>
+      </c>
+    </row>
+    <row>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">FL-04</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Launch - Terms &amp; Conditions link opens the terms page</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spider Solitaire Unity &gt; Launch</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Functional</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">High</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Close the page or tap Back.</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">The Terms &amp; Conditions card is still there. Do not tap Continue yet.</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Manual</t>
+        </is>
+      </c>
+    </row>
+    <row>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">FL-05</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Launch - Privacy Policy link opens the privacy page</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spider Solitaire Unity &gt; Launch</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Functional</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">High</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">On the same Terms &amp; Conditions card, tap Privacy Policy.</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">A privacy web page opens, not the Terms &amp; Conditions page.</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Manual</t>
+        </is>
+      </c>
+    </row>
+    <row>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">FL-05</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Launch - Privacy Policy link opens the privacy page</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spider Solitaire Unity &gt; Launch</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Functional</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">High</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">If Accept All Cookies appears, tap it and wait for the cookie banner to disappear.</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">The banner is gone and the Privacy Notice heading is fully visible.</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Manual</t>
+        </is>
+      </c>
+    </row>
+    <row>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">FL-05</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Launch - Privacy Policy link opens the privacy page</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spider Solitaire Unity &gt; Launch</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Functional</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">High</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Close the page or tap Back.</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">The Terms &amp; Conditions card is still there. Continue is checked separately in FL-02.</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Manual</t>
+        </is>
+      </c>
+    </row>
+    <row>
+      <c t="inlineStr">
+        <is>
           <t xml:space="preserve">MM-01</t>
         </is>
       </c>
@@ -4071,6 +4837,48 @@
     <row>
       <c t="inlineStr">
         <is>
+          <t xml:space="preserve">ST-01</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Statistics - Opens from the main menu</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spider Solitaire Unity &gt; Statistics</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Functional</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Medium</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">From the main menu, tap Stats.</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">The Statistics screen opens. The header reads Statistics. The main menu is gone.</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Manual</t>
+        </is>
+      </c>
+    </row>
+    <row>
+      <c t="inlineStr">
+        <is>
           <t xml:space="preserve">ST-03</t>
         </is>
       </c>
@@ -4155,6 +4963,90 @@
     <row>
       <c t="inlineStr">
         <is>
+          <t xml:space="preserve">ST-04</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Statistics - Back returns to the main menu</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spider Solitaire Unity &gt; Statistics</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Functional</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Medium</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">From Statistics, tap Back.</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">The main menu is showing.</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Manual</t>
+        </is>
+      </c>
+    </row>
+    <row>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">OP-01</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Options - Opens from the main menu</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spider Solitaire Unity &gt; Options</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Functional</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Medium</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">From the main menu, tap Options.</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">The Options screen opens. The main menu is gone.</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Manual</t>
+        </is>
+      </c>
+    </row>
+    <row>
+      <c t="inlineStr">
+        <is>
           <t xml:space="preserve">OP-03</t>
         </is>
       </c>
@@ -4491,6 +5383,48 @@
     <row>
       <c t="inlineStr">
         <is>
+          <t xml:space="preserve">HP-01</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Help - Opens on Introduction</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spider Solitaire Unity &gt; Help</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Functional</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Medium</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">From the main menu, tap Help.</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Help opens with the Introduction heading. The main menu is gone.</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Manual</t>
+        </is>
+      </c>
+    </row>
+    <row>
+      <c t="inlineStr">
+        <is>
           <t xml:space="preserve">HP-02</t>
         </is>
       </c>
@@ -4575,6 +5509,90 @@
     <row>
       <c t="inlineStr">
         <is>
+          <t xml:space="preserve">HP-03</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Help - Back returns to the main menu</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spider Solitaire Unity &gt; Help</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Functional</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Medium</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">From Help, tap Back.</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">The main menu is showing.</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Manual</t>
+        </is>
+      </c>
+    </row>
+    <row>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">AB-01</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">About - Opens from the About menu item</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spider Solitaire Unity &gt; About</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Functional</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Medium</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">From the main menu, tap About.</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">The About screen opens. You can see the copyright line.</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Manual</t>
+        </is>
+      </c>
+    </row>
+    <row>
+      <c t="inlineStr">
+        <is>
           <t xml:space="preserve">AB-03</t>
         </is>
       </c>
@@ -4827,6 +5845,48 @@
     <row>
       <c t="inlineStr">
         <is>
+          <t xml:space="preserve">MG-03</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">More Games - Back returns to the main menu</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spider Solitaire Unity &gt; More Games</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Functional</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Medium</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">From the More Games page, tap Back.</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">The main menu is showing.</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Manual</t>
+        </is>
+      </c>
+    </row>
+    <row>
+      <c t="inlineStr">
+        <is>
           <t xml:space="preserve">PL-01</t>
         </is>
       </c>
@@ -5877,6 +6937,48 @@
     <row>
       <c t="inlineStr">
         <is>
+          <t xml:space="preserve">VI-04</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Victory - Back returns to the main menu</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spider Solitaire Unity &gt; Victory</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Functional</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Medium</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">On Victory, tap the screen's own Back control — not New.</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">The main menu is showing. Leaving by Back leaves no game in progress.</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Manual</t>
+        </is>
+      </c>
+    </row>
+    <row>
+      <c t="inlineStr">
+        <is>
           <t xml:space="preserve">DL-01</t>
         </is>
       </c>
@@ -8008,6 +9110,48 @@
       <c t="inlineStr">
         <is>
           <t xml:space="preserve">Last Score is showing again.</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Manual</t>
+        </is>
+      </c>
+    </row>
+    <row>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">LS-05</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Last Score - Back returns to the main menu</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spider Solitaire Unity &gt; Last Score</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Functional</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Medium</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">From Last Score, tap Back until you reach the menu.</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">The main menu is showing.</t>
         </is>
       </c>
       <c t="inlineStr">

</xml_diff>

<commit_message>
Cover Contact Us both offline and online in run_all.
The suite still captures the no-network Helpshift redirect after Options, then comes online last to assert PeopleFun Support without letting ads interrupt earlier tests.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/testrail/spider_unity_cases.xlsx
+++ b/docs/testrail/spider_unity_cases.xlsx
@@ -4072,6 +4072,48 @@
     <row>
       <c t="inlineStr">
         <is>
+          <t xml:space="preserve">HS-02</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Options - Contact Us still leaves Options without internet</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spider Solitaire Unity &gt; Options</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Functional</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Medium</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. Turn Airplane Mode on and turn Wi-Fi off. Open Options and tap Contact Us.</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. You leave Options. The support page may show a no-connection or failed-load screen instead of PeopleFun Support. That is the case — the redirect still happened.</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Manual</t>
+        </is>
+      </c>
+    </row>
+    <row>
+      <c t="inlineStr">
+        <is>
           <t xml:space="preserve">RL-01</t>
         </is>
       </c>
@@ -9583,6 +9625,48 @@
     <row>
       <c t="inlineStr">
         <is>
+          <t xml:space="preserve">HS-02</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Options - Contact Us still leaves Options without internet</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spider Solitaire Unity &gt; Options</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Functional</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Medium</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Turn Airplane Mode on and turn Wi-Fi off. Open Options and tap Contact Us.</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">You leave Options. The support page may show a no-connection or failed-load screen instead of PeopleFun Support. That is the case — the redirect still happened.</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Manual</t>
+        </is>
+      </c>
+    </row>
+    <row>
+      <c t="inlineStr">
+        <is>
           <t xml:space="preserve">RL-01</t>
         </is>
       </c>

</xml_diff>

<commit_message>
Add negative Unity regression tests
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/testrail/spider_unity_cases.xlsx
+++ b/docs/testrail/spider_unity_cases.xlsx
@@ -1302,6 +1302,50 @@
     <row>
       <c t="inlineStr">
         <is>
+          <t xml:space="preserve">PL-04</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Play - Declining abandon stays on the picker</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spider Solitaire Unity &gt; Play</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Functional</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Medium</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. With a paused game, open Play and tap its difficulty again.
+2. Tap No.</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. An abandon confirmation appears.
+2. The new deal is cancelled. The difficulty picker remains open, the game table has not started, and the paused game has not been discarded.</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Manual</t>
+        </is>
+      </c>
+    </row>
+    <row>
+      <c t="inlineStr">
+        <is>
           <t xml:space="preserve">QA-02</t>
         </is>
       </c>
@@ -2626,6 +2670,50 @@
     <row>
       <c t="inlineStr">
         <is>
+          <t xml:space="preserve">RS-03</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Reset Statistics - Declining leaves scores alone</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spider Solitaire Unity &gt; Statistics</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Destructive</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Medium</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. Open Stats, scroll to Reset Statistics, and tap it.
+2. Tap No.</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. A reset confirmation appears.
+2. The confirmation closes, Statistics remains open, and the local scores are unchanged.</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Manual</t>
+        </is>
+      </c>
+    </row>
+    <row>
+      <c t="inlineStr">
+        <is>
           <t xml:space="preserve">CL-01</t>
         </is>
       </c>
@@ -3681,6 +3769,48 @@
       <c t="inlineStr">
         <is>
           <t xml:space="preserve">1. The main menu is showing.</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Manual</t>
+        </is>
+      </c>
+    </row>
+    <row>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">AF-01</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ad-free - No leaves you on About</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spider Solitaire Unity &gt; App Store / Mail</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Functional</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Medium</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. On About, tap ad free version and tap No on the confirmation.</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. The card closes. Spider stays in front on About and the App Store does not open.</t>
         </is>
       </c>
       <c t="inlineStr">
@@ -6055,6 +6185,90 @@
     <row>
       <c t="inlineStr">
         <is>
+          <t xml:space="preserve">PL-04</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Play - Declining abandon stays on the picker</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spider Solitaire Unity &gt; Play</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Functional</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Medium</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">With a paused game, open Play and tap its difficulty again.</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">An abandon confirmation appears.</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Manual</t>
+        </is>
+      </c>
+    </row>
+    <row>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">PL-04</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Play - Declining abandon stays on the picker</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spider Solitaire Unity &gt; Play</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Functional</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Medium</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tap No.</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">The new deal is cancelled. The difficulty picker remains open, the game table has not started, and the paused game has not been discarded.</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Manual</t>
+        </is>
+      </c>
+    </row>
+    <row>
+      <c t="inlineStr">
+        <is>
           <t xml:space="preserve">QA-02</t>
         </is>
       </c>
@@ -7819,6 +8033,90 @@
     <row>
       <c t="inlineStr">
         <is>
+          <t xml:space="preserve">RS-03</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Reset Statistics - Declining leaves scores alone</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spider Solitaire Unity &gt; Statistics</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Destructive</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Medium</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Open Stats, scroll to Reset Statistics, and tap it.</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">A reset confirmation appears.</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Manual</t>
+        </is>
+      </c>
+    </row>
+    <row>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">RS-03</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Reset Statistics - Declining leaves scores alone</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spider Solitaire Unity &gt; Statistics</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Destructive</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Medium</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tap No.</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">The confirmation closes, Statistics remains open, and the local scores are unchanged.</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Manual</t>
+        </is>
+      </c>
+    </row>
+    <row>
+      <c t="inlineStr">
+        <is>
           <t xml:space="preserve">CL-01</t>
         </is>
       </c>
@@ -9194,6 +9492,48 @@
       <c t="inlineStr">
         <is>
           <t xml:space="preserve">The main menu is showing.</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Manual</t>
+        </is>
+      </c>
+    </row>
+    <row>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">AF-01</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ad-free - No leaves you on About</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spider Solitaire Unity &gt; App Store / Mail</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Functional</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Medium</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">On About, tap ad free version and tap No on the confirmation.</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">The card closes. Spider stays in front on About and the App Store does not open.</t>
         </is>
       </c>
       <c t="inlineStr">

</xml_diff>

<commit_message>
Add TestFlight build installer to regression
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/testrail/spider_unity_cases.xlsx
+++ b/docs/testrail/spider_unity_cases.xlsx
@@ -284,6 +284,52 @@
     <row>
       <c t="inlineStr">
         <is>
+          <t xml:space="preserve">FL-06</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Launch - Latest odd TestFlight build installs</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spider Solitaire Unity &gt; Launch</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Functional</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">High</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. Open TestFlight and tap Spider / Spider Solitaire.
+2. Scroll to Previous Builds and tap it. Tap the top row.
+3. If that page's version in parentheses is odd, delete Spider if it is installed, then tap Install and wait. If it is even, stop.</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. The TestFlight page for this game is showing.
+2. The newest build's page is showing.
+3. The odd build installs. An even newest build leaves the existing Spider installation unchanged.</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Manual</t>
+        </is>
+      </c>
+    </row>
+    <row>
+      <c t="inlineStr">
+        <is>
           <t xml:space="preserve">MM-01</t>
         </is>
       </c>
@@ -4967,6 +5013,132 @@
     <row>
       <c t="inlineStr">
         <is>
+          <t xml:space="preserve">FL-06</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Launch - Latest odd TestFlight build installs</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spider Solitaire Unity &gt; Launch</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Functional</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">High</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Open TestFlight and tap Spider / Spider Solitaire.</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">The TestFlight page for this game is showing.</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Manual</t>
+        </is>
+      </c>
+    </row>
+    <row>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">FL-06</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Launch - Latest odd TestFlight build installs</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spider Solitaire Unity &gt; Launch</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Functional</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">High</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Scroll to Previous Builds and tap it. Tap the top row.</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">The newest build's page is showing.</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Manual</t>
+        </is>
+      </c>
+    </row>
+    <row>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">FL-06</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Launch - Latest odd TestFlight build installs</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spider Solitaire Unity &gt; Launch</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Functional</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">High</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">If that page's version in parentheses is odd, delete Spider if it is installed, then tap Install and wait. If it is even, stop.</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">The odd build installs. An even newest build leaves the existing Spider installation unchanged.</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Manual</t>
+        </is>
+      </c>
+    </row>
+    <row>
+      <c t="inlineStr">
+        <is>
           <t xml:space="preserve">MM-01</t>
         </is>
       </c>

</xml_diff>

<commit_message>
Report triggerAdPoints checks independently and drop the Resume menu-ad case.
A single failed check now fails its TA card without failing the parent, and TA-09 is retired because Resume no longer fires an interstitial.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/testrail/spider_unity_cases.xlsx
+++ b/docs/testrail/spider_unity_cases.xlsx
@@ -310,15 +310,15 @@
       <c t="inlineStr">
         <is>
           <t xml:space="preserve">1. Open TestFlight and tap Spider / Spider Solitaire.
-2. Scroll to Previous Builds and tap it. Tap the top row.
-3. If that page's version in parentheses is odd, delete Spider if it is installed, then tap Install and wait. If it is even, stop.</t>
+2. Scroll to Previous Builds and tap it. Review all individual build rows.
+3. If an odd build exists, delete Spider if it is installed, then tap Install for that exact row and wait. If all builds are even, stop.</t>
         </is>
       </c>
       <c t="inlineStr">
         <is>
           <t xml:space="preserve">1. The TestFlight page for this game is showing.
-2. The newest build's page is showing.
-3. The odd build installs. An even newest build leaves the existing Spider installation unchanged.</t>
+2. The greatest odd-numbered build is identified, regardless of where it appears in the list.
+3. The greatest odd build installs. An all-even list leaves the existing Spider installation unchanged.</t>
         </is>
       </c>
       <c t="inlineStr">
@@ -3528,48 +3528,6 @@
     <row>
       <c t="inlineStr">
         <is>
-          <t xml:space="preserve">TA-09</t>
-        </is>
-      </c>
-      <c t="inlineStr">
-        <is>
-          <t xml:space="preserve">Ads - Starting a game after 30s on the menu shows an ad</t>
-        </is>
-      </c>
-      <c t="inlineStr">
-        <is>
-          <t xml:space="preserve">Spider Solitaire Unity &gt; Ads</t>
-        </is>
-      </c>
-      <c t="inlineStr">
-        <is>
-          <t xml:space="preserve">Functional</t>
-        </is>
-      </c>
-      <c t="inlineStr">
-        <is>
-          <t xml:space="preserve">High</t>
-        </is>
-      </c>
-      <c t="inlineStr">
-        <is>
-          <t xml:space="preserve">1. Leave a table with Back after more than 30 seconds, close that ad onto the menu, stay on the menu more than 30 seconds, then resume or deal.</t>
-        </is>
-      </c>
-      <c t="inlineStr">
-        <is>
-          <t xml:space="preserve">1. An ad plays as you enter the game. This is the menu wait, not the same as the leave-game ad.</t>
-        </is>
-      </c>
-      <c t="inlineStr">
-        <is>
-          <t xml:space="preserve">Manual</t>
-        </is>
-      </c>
-    </row>
-    <row>
-      <c t="inlineStr">
-        <is>
           <t xml:space="preserve">TA-10</t>
         </is>
       </c>
@@ -3727,7 +3685,7 @@
       </c>
       <c t="inlineStr">
         <is>
-          <t xml:space="preserve">1. Game Center opens, headed Leaderboards.
+          <t xml:space="preserve">1. Game Center opens, headed Leaderboards. If a notice card appears instead (scores may take a little time to upload), tap OK — Leaderboards opens from that, do not tap the link again.
 2. Last Score is showing again.</t>
         </is>
       </c>
@@ -3771,7 +3729,7 @@
       </c>
       <c t="inlineStr">
         <is>
-          <t xml:space="preserve">1. Game Center opens, headed Achievements.
+          <t xml:space="preserve">1. Game Center opens, headed Achievements. If the same notice card appears, tap OK — Achievements opens from that, do not tap the link again.
 2. Last Score is showing again.</t>
         </is>
       </c>
@@ -5080,12 +5038,12 @@
       </c>
       <c t="inlineStr">
         <is>
-          <t xml:space="preserve">Scroll to Previous Builds and tap it. Tap the top row.</t>
-        </is>
-      </c>
-      <c t="inlineStr">
-        <is>
-          <t xml:space="preserve">The newest build's page is showing.</t>
+          <t xml:space="preserve">Scroll to Previous Builds and tap it. Review all individual build rows.</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">The greatest odd-numbered build is identified, regardless of where it appears in the list.</t>
         </is>
       </c>
       <c t="inlineStr">
@@ -5122,12 +5080,12 @@
       </c>
       <c t="inlineStr">
         <is>
-          <t xml:space="preserve">If that page's version in parentheses is odd, delete Spider if it is installed, then tap Install and wait. If it is even, stop.</t>
-        </is>
-      </c>
-      <c t="inlineStr">
-        <is>
-          <t xml:space="preserve">The odd build installs. An even newest build leaves the existing Spider installation unchanged.</t>
+          <t xml:space="preserve">If an odd build exists, delete Spider if it is installed, then tap Install for that exact row and wait. If all builds are even, stop.</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">The greatest odd build installs. An all-even list leaves the existing Spider installation unchanged.</t>
         </is>
       </c>
       <c t="inlineStr">
@@ -9297,12 +9255,12 @@
     <row>
       <c t="inlineStr">
         <is>
-          <t xml:space="preserve">TA-09</t>
-        </is>
-      </c>
-      <c t="inlineStr">
-        <is>
-          <t xml:space="preserve">Ads - Starting a game after 30s on the menu shows an ad</t>
+          <t xml:space="preserve">TA-10</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ads - Over 30s on the table, FAQ shows an ad</t>
         </is>
       </c>
       <c t="inlineStr">
@@ -9322,48 +9280,6 @@
       </c>
       <c t="inlineStr">
         <is>
-          <t xml:space="preserve">Leave a table with Back after more than 30 seconds, close that ad onto the menu, stay on the menu more than 30 seconds, then resume or deal.</t>
-        </is>
-      </c>
-      <c t="inlineStr">
-        <is>
-          <t xml:space="preserve">An ad plays as you enter the game. This is the menu wait, not the same as the leave-game ad.</t>
-        </is>
-      </c>
-      <c t="inlineStr">
-        <is>
-          <t xml:space="preserve">Manual</t>
-        </is>
-      </c>
-    </row>
-    <row>
-      <c t="inlineStr">
-        <is>
-          <t xml:space="preserve">TA-10</t>
-        </is>
-      </c>
-      <c t="inlineStr">
-        <is>
-          <t xml:space="preserve">Ads - Over 30s on the table, FAQ shows an ad</t>
-        </is>
-      </c>
-      <c t="inlineStr">
-        <is>
-          <t xml:space="preserve">Spider Solitaire Unity &gt; Ads</t>
-        </is>
-      </c>
-      <c t="inlineStr">
-        <is>
-          <t xml:space="preserve">Functional</t>
-        </is>
-      </c>
-      <c t="inlineStr">
-        <is>
-          <t xml:space="preserve">High</t>
-        </is>
-      </c>
-      <c t="inlineStr">
-        <is>
           <t xml:space="preserve">Stay on the table more than 30 seconds. Open the in-game menu and tap FAQ.</t>
         </is>
       </c>
@@ -9495,7 +9411,7 @@
       </c>
       <c t="inlineStr">
         <is>
-          <t xml:space="preserve">Game Center opens, headed Leaderboards.</t>
+          <t xml:space="preserve">Game Center opens, headed Leaderboards. If a notice card appears instead (scores may take a little time to upload), tap OK — Leaderboards opens from that, do not tap the link again.</t>
         </is>
       </c>
       <c t="inlineStr">
@@ -9579,7 +9495,7 @@
       </c>
       <c t="inlineStr">
         <is>
-          <t xml:space="preserve">Game Center opens, headed Achievements.</t>
+          <t xml:space="preserve">Game Center opens, headed Achievements. If the same notice card appears, tap OK — Achievements opens from that, do not tap the link again.</t>
         </is>
       </c>
       <c t="inlineStr">

</xml_diff>